<commit_message>
upd docs && added new ones
</commit_message>
<xml_diff>
--- a/EntrepreneurialWorkshop/UsefulMaterials/Yu-Ri_Track_card.xlsx
+++ b/EntrepreneurialWorkshop/UsefulMaterials/Yu-Ri_Track_card.xlsx
@@ -5,16 +5,17 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\МАРГАРИТА\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\HSE\HSE-FCS-SE-2-course\EntrepreneurialWorkshop\UsefulMaterials\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4B1B26AB-85C9-4300-B7AC-3E674C4BE014}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E95FD3C4-FBF1-476C-BBF4-0B4E558886E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="легенда" sheetId="1" r:id="rId1"/>
     <sheet name="неделя 1" sheetId="2" r:id="rId2"/>
+    <sheet name="Лист1" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -99,9 +100,6 @@
   </si>
   <si>
     <t>помогаем клиентам типа юристов частной практики, ИТ-стартапов без юриста в штате и финансовых компаний с большим объемом договоров</t>
-  </si>
-  <si>
-    <t>13.04 - 19.04</t>
   </si>
   <si>
     <r>
@@ -277,6 +275,9 @@
   </si>
   <si>
     <t>Продление → Рекомендация</t>
+  </si>
+  <si>
+    <t>25.04 - 20.05</t>
   </si>
 </sst>
 </file>
@@ -472,18 +473,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -491,12 +480,6 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -511,12 +494,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -526,10 +503,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -549,6 +522,34 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -823,11 +824,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="20" t="s">
-        <v>22</v>
+      <c r="B1" s="16" t="s">
+        <v>59</v>
       </c>
       <c r="C1" s="1"/>
       <c r="G1" s="1"/>
@@ -855,14 +856,14 @@
       <c r="O2" s="1"/>
     </row>
     <row r="3" spans="1:15" ht="36" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="35" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
-      <c r="D3" s="31"/>
-      <c r="E3" s="31"/>
-      <c r="F3" s="31"/>
+      <c r="B3" s="36"/>
+      <c r="C3" s="36"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
       <c r="G3" s="1"/>
       <c r="H3" s="1"/>
       <c r="I3" s="1"/>
@@ -889,7 +890,7 @@
     </row>
     <row r="5" spans="1:15" ht="13.2" x14ac:dyDescent="0.25">
       <c r="A5" s="14" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
@@ -921,7 +922,7 @@
     </row>
     <row r="7" spans="1:15" ht="66" x14ac:dyDescent="0.25">
       <c r="A7" s="14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B7" s="1"/>
       <c r="C7" s="1"/>
@@ -937,7 +938,7 @@
     </row>
     <row r="8" spans="1:15" ht="79.2" x14ac:dyDescent="0.25">
       <c r="A8" s="14" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -953,7 +954,7 @@
     </row>
     <row r="9" spans="1:15" ht="66" x14ac:dyDescent="0.25">
       <c r="A9" s="14" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -982,30 +983,30 @@
       <c r="O10" s="1"/>
     </row>
     <row r="11" spans="1:15" ht="29.25" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A11" s="17" t="s">
+      <c r="A11" s="37" t="s">
         <v>4</v>
       </c>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
-      <c r="F11" s="25"/>
-      <c r="G11" s="25"/>
-      <c r="H11" s="25"/>
-      <c r="I11" s="25"/>
-      <c r="J11" s="25"/>
-      <c r="K11" s="25"/>
-      <c r="L11" s="37"/>
-      <c r="M11" s="37"/>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="19"/>
+      <c r="E11" s="19"/>
+      <c r="F11" s="19"/>
+      <c r="G11" s="19"/>
+      <c r="H11" s="19"/>
+      <c r="I11" s="19"/>
+      <c r="J11" s="19"/>
+      <c r="K11" s="19"/>
+      <c r="L11" s="27"/>
+      <c r="M11" s="27"/>
       <c r="N11" s="1"/>
       <c r="O11" s="1"/>
     </row>
     <row r="12" spans="1:15" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A12" s="27" t="s">
+      <c r="A12" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B12" s="36" t="s">
-        <v>27</v>
+      <c r="B12" s="26" t="s">
+        <v>26</v>
       </c>
       <c r="C12" s="9"/>
       <c r="D12" s="9"/>
@@ -1022,28 +1023,28 @@
       <c r="O12" s="1"/>
     </row>
     <row r="13" spans="1:15" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A13" s="32"/>
-      <c r="B13" s="32"/>
-      <c r="C13" s="32"/>
-      <c r="D13" s="32"/>
-      <c r="E13" s="32"/>
-      <c r="F13" s="32"/>
-      <c r="G13" s="32"/>
-      <c r="H13" s="32"/>
-      <c r="I13" s="32"/>
-      <c r="J13" s="32"/>
-      <c r="K13" s="32"/>
+      <c r="A13" s="24"/>
+      <c r="B13" s="24"/>
+      <c r="C13" s="24"/>
+      <c r="D13" s="24"/>
+      <c r="E13" s="24"/>
+      <c r="F13" s="24"/>
+      <c r="G13" s="24"/>
+      <c r="H13" s="24"/>
+      <c r="I13" s="24"/>
+      <c r="J13" s="24"/>
+      <c r="K13" s="24"/>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
       <c r="N13" s="1"/>
       <c r="O13" s="1"/>
     </row>
     <row r="14" spans="1:15" ht="13.8" x14ac:dyDescent="0.3">
-      <c r="A14" s="27" t="s">
+      <c r="A14" s="21" t="s">
         <v>6</v>
       </c>
-      <c r="B14" s="36" t="s">
-        <v>28</v>
+      <c r="B14" s="26" t="s">
+        <v>27</v>
       </c>
       <c r="C14" s="9"/>
       <c r="D14" s="9"/>
@@ -1074,14 +1075,14 @@
       <c r="O15" s="1"/>
     </row>
     <row r="16" spans="1:15" ht="31.5" customHeight="1" x14ac:dyDescent="0.4">
-      <c r="A16" s="22" t="s">
+      <c r="A16" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
+      <c r="B16" s="40"/>
+      <c r="C16" s="40"/>
+      <c r="D16" s="22"/>
+      <c r="E16" s="22"/>
+      <c r="F16" s="22"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
       <c r="I16" s="1"/>
@@ -1093,12 +1094,12 @@
       <c r="O16" s="1"/>
     </row>
     <row r="17" spans="1:17" ht="13.2" x14ac:dyDescent="0.25">
-      <c r="A17" s="32"/>
-      <c r="B17" s="32"/>
-      <c r="C17" s="32"/>
-      <c r="D17" s="32"/>
-      <c r="E17" s="32"/>
-      <c r="F17" s="32"/>
+      <c r="A17" s="24"/>
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
@@ -1110,14 +1111,14 @@
       <c r="O17" s="1"/>
     </row>
     <row r="18" spans="1:17" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="41" t="s">
         <v>8</v>
       </c>
-      <c r="B18" s="29"/>
-      <c r="C18" s="29"/>
-      <c r="D18" s="35"/>
-      <c r="E18" s="35"/>
-      <c r="F18" s="35"/>
+      <c r="B18" s="42"/>
+      <c r="C18" s="42"/>
+      <c r="D18" s="25"/>
+      <c r="E18" s="25"/>
+      <c r="F18" s="25"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -1129,20 +1130,20 @@
       <c r="O18" s="1"/>
     </row>
     <row r="19" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="18" t="s">
         <v>9</v>
       </c>
-      <c r="B19" s="24" t="s">
+      <c r="B19" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="C19" s="24" t="s">
+      <c r="C19" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="D19" s="24" t="s">
+      <c r="D19" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
+      <c r="E19" s="18"/>
+      <c r="F19" s="18"/>
       <c r="G19" s="6"/>
       <c r="H19" s="6"/>
       <c r="I19" s="6"/>
@@ -1154,20 +1155,20 @@
       <c r="O19" s="6"/>
     </row>
     <row r="20" spans="1:17" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A20" s="26" t="s">
-        <v>29</v>
+      <c r="A20" s="20" t="s">
+        <v>28</v>
       </c>
-      <c r="B20" s="26" t="s">
+      <c r="B20" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C20" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="26" t="s">
+      <c r="D20" s="20" t="s">
         <v>33</v>
       </c>
-      <c r="D20" s="26" t="s">
-        <v>34</v>
-      </c>
-      <c r="E20" s="26"/>
-      <c r="F20" s="26"/>
+      <c r="E20" s="20"/>
+      <c r="F20" s="20"/>
       <c r="G20" s="6"/>
       <c r="H20" s="6"/>
       <c r="I20" s="6"/>
@@ -1180,7 +1181,7 @@
     </row>
     <row r="21" spans="1:17" ht="52.8" x14ac:dyDescent="0.25">
       <c r="A21" s="10" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B21" s="10" t="s">
         <v>13</v>
@@ -1189,7 +1190,7 @@
         <v>14</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" s="10"/>
       <c r="F21" s="10"/>
@@ -1205,16 +1206,16 @@
     </row>
     <row r="22" spans="1:17" ht="66" x14ac:dyDescent="0.25">
       <c r="A22" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B22" s="11" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" s="11" t="s">
         <v>36</v>
       </c>
-      <c r="C22" s="11" t="s">
+      <c r="D22" s="11" t="s">
         <v>37</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>38</v>
       </c>
       <c r="E22" s="11"/>
       <c r="F22" s="11"/>
@@ -1248,10 +1249,10 @@
       </c>
       <c r="B24" s="34"/>
       <c r="C24" s="34"/>
-      <c r="D24" s="38"/>
-      <c r="E24" s="38"/>
-      <c r="F24" s="38"/>
-      <c r="G24" s="39"/>
+      <c r="D24" s="28"/>
+      <c r="E24" s="28"/>
+      <c r="F24" s="28"/>
+      <c r="G24" s="29"/>
       <c r="H24" s="1"/>
       <c r="I24" s="1"/>
       <c r="J24" s="1"/>
@@ -1281,7 +1282,7 @@
         <v>17</v>
       </c>
       <c r="G25" s="12" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="H25" s="1"/>
       <c r="I25" s="1"/>
@@ -1295,26 +1296,26 @@
       <c r="Q25" s="1"/>
     </row>
     <row r="26" spans="1:17" ht="52.8" x14ac:dyDescent="0.25">
-      <c r="A26" s="41">
+      <c r="A26" s="31">
         <v>1</v>
       </c>
-      <c r="B26" s="40" t="s">
-        <v>29</v>
+      <c r="B26" s="30" t="s">
+        <v>28</v>
       </c>
-      <c r="C26" s="42" t="s">
-        <v>50</v>
+      <c r="C26" s="32" t="s">
+        <v>49</v>
       </c>
-      <c r="D26" s="42" t="s">
+      <c r="D26" s="32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="E26" s="42" t="s">
+      <c r="F26" s="32" t="s">
         <v>40</v>
       </c>
-      <c r="F26" s="42" t="s">
-        <v>41</v>
-      </c>
-      <c r="G26" s="21" t="s">
-        <v>43</v>
+      <c r="G26" s="17" t="s">
+        <v>42</v>
       </c>
       <c r="H26" s="1"/>
       <c r="I26" s="1"/>
@@ -1330,22 +1331,22 @@
         <v>2</v>
       </c>
       <c r="B27" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="C27" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="D27" s="13" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="D27" s="13" t="s">
+      <c r="E27" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="E27" s="13" t="s">
-        <v>46</v>
-      </c>
       <c r="F27" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
@@ -1361,22 +1362,22 @@
         <v>3</v>
       </c>
       <c r="B28" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C28" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="D28" s="13" t="s">
         <v>52</v>
       </c>
-      <c r="D28" s="13" t="s">
+      <c r="E28" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="E28" s="13" t="s">
+      <c r="F28" s="13" t="s">
         <v>54</v>
       </c>
-      <c r="F28" s="13" t="s">
+      <c r="G28" s="9" t="s">
         <v>55</v>
-      </c>
-      <c r="G28" s="9" t="s">
-        <v>56</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
@@ -1392,22 +1393,22 @@
         <v>4</v>
       </c>
       <c r="B29" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C29" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D29" s="13" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="E29" s="13" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F29" s="13" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
@@ -14883,4 +14884,13 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DF2013F-BFAB-4DA9-B435-627C95253DA5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="13.2" x14ac:dyDescent="0.25"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>